<commit_message>
Simplificacion parcial con clases
</commit_message>
<xml_diff>
--- a/Pasta_Biwenger_Portatil_Gris.xlsx
+++ b/Pasta_Biwenger_Portatil_Gris.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juliu\Documents\biwenger\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5A8BF2C-7037-4E0D-98F1-4E5E9D2AFCFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{974DAC48-D3B4-48E6-BC09-CE758F82E04E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="995" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="995" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Automate" sheetId="1" r:id="rId1"/>
@@ -3152,7 +3152,7 @@
       </c>
       <c r="L1" s="10">
         <f ca="1">TODAY()</f>
-        <v>45937</v>
+        <v>45938</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="L1" s="10">
         <f ca="1">TODAY()</f>
-        <v>45937</v>
+        <v>45938</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -4489,7 +4489,7 @@
       </c>
       <c r="L1" s="6">
         <f ca="1">TODAY()</f>
-        <v>45937</v>
+        <v>45938</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -5223,7 +5223,7 @@
       </c>
       <c r="L1" s="6">
         <f ca="1">TODAY()</f>
-        <v>45937</v>
+        <v>45938</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -10925,7 +10925,7 @@
       </c>
       <c r="L1" s="6">
         <f ca="1">TODAY()</f>
-        <v>45937</v>
+        <v>45938</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -11554,7 +11554,7 @@
       </c>
       <c r="L1" s="10">
         <f ca="1">TODAY()</f>
-        <v>45937</v>
+        <v>45938</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -12182,7 +12182,7 @@
       </c>
       <c r="J1" s="6">
         <f ca="1">TODAY()</f>
-        <v>45937</v>
+        <v>45938</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -12925,7 +12925,7 @@
       </c>
       <c r="L1" s="10">
         <f ca="1">TODAY()</f>
-        <v>45937</v>
+        <v>45938</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -13578,7 +13578,7 @@
       </c>
       <c r="L1" s="10">
         <f ca="1">TODAY()</f>
-        <v>45937</v>
+        <v>45938</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -14173,13 +14173,11 @@
       </c>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="F28"/>
       <c r="J28" s="5" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="F29"/>
       <c r="J29" t="s">
         <v>76</v>
       </c>
@@ -14307,7 +14305,7 @@
       </c>
       <c r="L1" s="10">
         <f ca="1">TODAY()</f>
-        <v>45937</v>
+        <v>45938</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -14990,7 +14988,7 @@
       </c>
       <c r="L1" s="10">
         <f ca="1">TODAY()</f>
-        <v>45937</v>
+        <v>45938</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -15646,7 +15644,7 @@
       </c>
       <c r="L1" s="10">
         <f ca="1">TODAY()</f>
-        <v>45937</v>
+        <v>45938</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>